<commit_message>
working inventory and unvax child start
</commit_message>
<xml_diff>
--- a/horizon excursion/15 years - starting unvax children/Demand_Scenarios_updated.xlsx
+++ b/horizon excursion/15 years - starting unvax children/Demand_Scenarios_updated.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/horizon excursion/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/horizon excursion/15 years - starting unvax children/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="131" documentId="13_ncr:1_{846A7131-5717-4B26-8D95-A495C589879C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F21E8C4C-644C-438B-9B9B-F71420E1B09E}"/>
+  <xr:revisionPtr revIDLastSave="167" documentId="13_ncr:1_{846A7131-5717-4B26-8D95-A495C589879C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{28861739-AF0C-4140-8143-71574242E728}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="3" activeTab="4" xr2:uid="{4E5F4A35-5A78-441E-8AE9-B1CCE3EF1506}"/>
+    <workbookView xWindow="13550" yWindow="-110" windowWidth="38620" windowHeight="21100" firstSheet="2" activeTab="4" xr2:uid="{4E5F4A35-5A78-441E-8AE9-B1CCE3EF1506}"/>
   </bookViews>
   <sheets>
     <sheet name="vaccine-producer list" sheetId="70" r:id="rId1"/>
@@ -1652,9 +1652,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1692,7 +1692,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1798,7 +1798,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1940,7 +1940,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -37305,11 +37305,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E6D5A8F-84A7-44FF-8A0A-25164FF49045}">
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:P42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="11" width="13.7109375" customWidth="1"/>
     <col min="12" max="12" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
@@ -38027,24 +38027,81 @@
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B16" s="71"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="51"/>
       <c r="B17" s="72"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="69"/>
       <c r="B18" s="72"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="69"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B20" s="69"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D31" s="50"/>
+      <c r="E31" s="51"/>
+      <c r="H31" s="69"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D32" s="50"/>
+      <c r="E32" s="51"/>
+      <c r="H32" s="69"/>
+    </row>
+    <row r="33" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D33" s="50"/>
+      <c r="E33" s="51"/>
+      <c r="H33" s="69"/>
+    </row>
+    <row r="34" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D34" s="50"/>
+      <c r="E34" s="51"/>
+      <c r="H34" s="69"/>
+    </row>
+    <row r="35" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D35" s="50"/>
+      <c r="E35" s="51"/>
+      <c r="H35" s="69"/>
+    </row>
+    <row r="36" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D36" s="50"/>
+      <c r="E36" s="51"/>
+      <c r="H36" s="69"/>
+    </row>
+    <row r="37" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D37" s="50"/>
+      <c r="E37" s="51"/>
+      <c r="H37" s="69"/>
+    </row>
+    <row r="38" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D38" s="50"/>
+      <c r="E38" s="51"/>
+      <c r="H38" s="69"/>
+    </row>
+    <row r="39" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D39" s="50"/>
+      <c r="E39" s="51"/>
+      <c r="H39" s="69"/>
+    </row>
+    <row r="40" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="E40" s="51"/>
+      <c r="H40" s="69"/>
+    </row>
+    <row r="41" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="E41" s="51"/>
+      <c r="H41" s="69"/>
+    </row>
+    <row r="42" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="E42" s="51"/>
+      <c r="H42" s="69"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>